<commit_message>
Checkpoint SBG-v4 pipeline and 47-verse workbook
</commit_message>
<xml_diff>
--- a/data/Bhagavad_Gita_Content_Master_Chapter1_Verses1-5.xlsx
+++ b/data/Bhagavad_Gita_Content_Master_Chapter1_Verses1-5.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Master_V1-5" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Content_Master_V1-5" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Content_Master_V1-5'!$A$1:$T$6</definedName>
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:X6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -562,6 +562,26 @@
       <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Upload Status</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Scene 1 Narration</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Scene 2 Narration</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Scene 3 Narration</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Scene 4 Narration</t>
         </is>
       </c>
     </row>
@@ -678,6 +698,26 @@
           <t>Pending</t>
         </is>
       </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>We are reciting Shree Bhagavad Gita, Chapter 1, Shloka 1.</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>धृतराष्ट्र उवाच । धर्मक्षेत्रे कुरुक्षेत्रे समवेता युयुत्सवः । मामकाः पाण्डवाश्चैव किमकुर्वत सञ्जय ॥</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Dhritarashtra asks Sanjaya what happened when the Kauravas and Pandavas gathered at Kurukshetra, ready for battle.</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Before reacting to conflict, pause and seek clarity. Sometimes, wisdom begins simply by choosing to see clearly.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">

</xml_diff>